<commit_message>
Remove attribute children for correct hierarchy
</commit_message>
<xml_diff>
--- a/inbox-excel-vocabs/voc4cat.xlsx
+++ b/inbox-excel-vocabs/voc4cat.xlsx
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3425" uniqueCount="1935">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3426" uniqueCount="1935">
   <si>
     <t xml:space="preserve">Template version</t>
   </si>
@@ -5896,7 +5896,6 @@
 voc4cat:0007261 (peak area),
 voc4cat:0007262 (membrane thickness),
 voc4cat:0007263 (total faradaic efficiency),
-voc4cat:0008084 (detector dead time),
 voc4cat:0008085 (dead time correction),
 voc4cat:0008086 (fluorescence yield),
 voc4cat:0008087 (absorbance),
@@ -5904,11 +5903,6 @@
 voc4cat:0008089 (absorbance of the sample),
 voc4cat:0008090 (manual energy shift),
 voc4cat:0008091 (fluorescence signal),
-voc4cat:0008092 (incoming count rate),
-voc4cat:0008093 (outgoing count rate),
-voc4cat:0008094 (trigger live time),
-voc4cat:0008095 (effective measurement time),
-voc4cat:0008096 (total measurement time),
 voc4cat:0008097 (X-ray photon energy),
 voc4cat:0008099 (dead time),
 voc4cat:0008100 (detector performance measure)
@@ -7380,9 +7374,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>579240</xdr:colOff>
+      <xdr:colOff>578520</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>131760</xdr:rowOff>
+      <xdr:rowOff>131040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7396,8 +7390,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1377360" y="304920"/>
-          <a:ext cx="5910120" cy="1541520"/>
+          <a:off x="1378440" y="304920"/>
+          <a:ext cx="5909400" cy="1540800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7472,7 +7466,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A11:L32"/>
-  <sheetFormatPr defaultColWidth="12.6015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="2" style="1" width="12.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9.28"/>
@@ -7660,7 +7654,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J1149"/>
-  <sheetFormatPr defaultColWidth="12.6015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="16"/>
@@ -10343,7 +10337,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D994"/>
-  <sheetFormatPr defaultColWidth="12.6015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="72.7"/>
@@ -11510,7 +11504,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I527"/>
-  <sheetFormatPr defaultColWidth="12.6015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.7"/>
@@ -22963,7 +22957,7 @@
       </c>
       <c r="I480" s="34"/>
     </row>
-    <row r="481" customFormat="false" ht="1706.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="481" customFormat="false" ht="1624.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A481" s="34" t="s">
         <v>1734</v>
       </c>
@@ -23387,7 +23381,7 @@
         <v>1742</v>
       </c>
     </row>
-    <row r="500" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="500" customFormat="false" ht="80.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A500" s="34" t="s">
         <v>1807</v>
       </c>
@@ -23406,6 +23400,9 @@
       <c r="F500" s="0"/>
       <c r="G500" s="35" t="s">
         <v>1810</v>
+      </c>
+      <c r="H500" s="1" t="s">
+        <v>1742</v>
       </c>
     </row>
     <row r="501" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -23919,7 +23916,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F461"/>
-  <sheetFormatPr defaultColWidth="12.6015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="1" style="1" width="42.71"/>
   </cols>
@@ -24694,7 +24691,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E28"/>
-  <sheetFormatPr defaultColWidth="12.6015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40.7"/>
@@ -24972,7 +24969,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B31"/>
-  <sheetFormatPr defaultColWidth="12.6015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6171875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="60.72"/>

</xml_diff>